<commit_message>
Scores from Score_Card_5: WS final, WD semifinal 2, MS quarterfinal 3, corrected match 57
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KpjSian9KihxBdn7Md9Nh1
</commit_message>
<xml_diff>
--- a/scores/Score_Card.xlsx
+++ b/scores/Score_Card.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliakber/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EECABB7-CFB9-A546-9D28-90C85727EC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A03DEF97-D341-7948-99A5-F5175C407AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="7" xr2:uid="{80F890F9-808C-4260-AFEB-091B93DC4636}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16960" activeTab="6" xr2:uid="{80F890F9-808C-4260-AFEB-091B93DC4636}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -1119,7 +1119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1281,14 +1281,12 @@
     <xf numFmtId="0" fontId="11" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1302,14 +1300,17 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6309,7 +6310,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="9" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B9" s="41" t="s">
         <v>10</v>
       </c>
@@ -6608,7 +6609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B15" s="41" t="s">
         <v>10</v>
       </c>
@@ -6658,7 +6659,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B16" s="41" t="s">
         <v>10</v>
       </c>
@@ -6958,7 +6959,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="22" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B22" s="41" t="s">
         <v>26</v>
       </c>
@@ -7858,7 +7859,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="40" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B40" s="41" t="s">
         <v>31</v>
       </c>
@@ -8835,27 +8836,27 @@
       </c>
       <c r="J59" s="40" t="str">
         <f t="shared" si="10"/>
-        <v>Mamta + Rithu</v>
+        <v>Vaishnavi M + Keerthana</v>
       </c>
       <c r="K59" s="45" t="s">
-        <v>127</v>
+        <v>106</v>
       </c>
       <c r="L59" s="40" t="str">
         <f t="shared" si="6"/>
-        <v>Team 3</v>
+        <v>Team 2</v>
       </c>
       <c r="M59" s="39"/>
       <c r="N59" s="14">
         <f t="shared" si="7"/>
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="O59" s="14">
         <f t="shared" si="8"/>
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="P59" s="14">
         <f t="shared" si="9"/>
-        <v>-7</v>
+        <v>7</v>
       </c>
     </row>
     <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
@@ -9108,7 +9109,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B65" s="41" t="s">
         <v>37</v>
       </c>
@@ -9408,7 +9409,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B71" s="41" t="s">
         <v>37</v>
       </c>
@@ -9758,7 +9759,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="78" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B78" s="41" t="s">
         <v>40</v>
       </c>
@@ -10308,7 +10309,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B89" s="41" t="s">
         <v>43</v>
       </c>
@@ -10809,7 +10810,7 @@
         <v>-15</v>
       </c>
     </row>
-    <row r="99" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B99" s="41" t="s">
         <v>43</v>
       </c>
@@ -11108,7 +11109,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B105" s="41" t="s">
         <v>46</v>
       </c>
@@ -11275,8 +11276,10 @@
     </row>
   </sheetData>
   <autoFilter ref="B2:M107" xr:uid="{8D08637B-F719-49C8-8CD0-A0482E45DECD}">
-    <filterColumn colId="10">
-      <filters blank="1"/>
+    <filterColumn colId="5">
+      <filters>
+        <filter val="Women's Doubles"/>
+      </filters>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="J3:K92 K93 J94:K102 J103:J107 K103:K112">
@@ -11457,7 +11460,7 @@
       </c>
       <c r="C6" s="11">
         <f>'Points Table'!D27</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" s="11">
         <f>'Points Table'!D37</f>
@@ -11481,11 +11484,11 @@
       </c>
       <c r="I6" s="12">
         <f t="shared" ref="I6:I10" si="0">SUM(B6:H6)</f>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J6" s="55">
         <f>'Points Table'!G7</f>
-        <v>-47</v>
+        <v>-33</v>
       </c>
       <c r="K6" s="12">
         <f t="shared" ref="K6:K10" si="1">1+COUNTIF($I$5:$I$10,"&gt;"&amp;I6)+COUNTIFS($I$5:$I$10,I6,$J$5:$J$10,"&gt;"&amp;J6)+COUNTIFS($I$5:$I$10,I6,$J$5:$J$10,J6,$A$5:$A$10,"&lt;"&amp;A6)</f>
@@ -11506,7 +11509,7 @@
       </c>
       <c r="C7" s="11">
         <f>'Points Table'!D28</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" s="11">
         <f>'Points Table'!D38</f>
@@ -11530,11 +11533,11 @@
       </c>
       <c r="I7" s="12">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J7" s="55">
         <f>'Points Table'!G8</f>
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="K7" s="12">
         <f t="shared" si="1"/>
@@ -11768,11 +11771,11 @@
       </c>
       <c r="C15" s="9">
         <f>IF(B15="","",_xlfn.XLOOKUP(A15,$K$5:$K$10,$I$5:$I$10,""))</f>
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D15" s="56">
         <f>IF(B15="","",_xlfn.XLOOKUP(A15,$K$5:$K$10,$J$5:$J$10,""))</f>
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -11818,11 +11821,11 @@
       </c>
       <c r="C17" s="9">
         <f t="shared" si="2"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D17" s="56">
         <f t="shared" si="3"/>
-        <v>-47</v>
+        <v>-33</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -11880,7 +11883,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AAE4D3B-3905-4287-A120-83F138B0B077}">
-  <dimension ref="B2:L97"/>
+  <dimension ref="B2:M97"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="14" customWidth="1"/>
@@ -12265,7 +12268,7 @@
       <c r="K16" s="64"/>
       <c r="L16" s="18"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="17" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B17" s="37" t="s">
         <v>241</v>
       </c>
@@ -12280,7 +12283,7 @@
       <c r="K17" s="37"/>
       <c r="L17" s="37"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B18" s="16" t="s">
         <v>131</v>
       </c>
@@ -12313,7 +12316,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B19" s="19" t="s">
         <v>2</v>
       </c>
@@ -12354,21 +12357,21 @@
         <v>105</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B20" s="19" t="s">
         <v>3</v>
       </c>
       <c r="C20" s="20">
         <f>'Points Table'!D27</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D20" s="52">
         <f>'Points Table'!G27</f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E20" s="57">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" s="19" t="str">
         <f>IF(COUNTIFS('Shuffled Matches'!$G$3:$G$107,"Women's Doubles",'Shuffled Matches'!$K$3:$K$107,"&lt;&gt;")=0,"Pending",IF(E20&lt;=4,"Top 4","Eliminated"))</f>
@@ -12392,20 +12395,20 @@
       </c>
       <c r="L20" s="17">
         <f>'Points Table'!E27</f>
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.15">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B21" s="19" t="s">
         <v>63</v>
       </c>
       <c r="C21" s="20">
         <f>'Points Table'!D28</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D21" s="52">
         <f>'Points Table'!G28</f>
-        <v>-10</v>
+        <v>-24</v>
       </c>
       <c r="E21" s="57">
         <f t="shared" si="1"/>
@@ -12421,22 +12424,23 @@
       </c>
       <c r="I21" s="22" t="str">
         <f>IF(COUNTIFS('Shuffled Matches'!$G$3:$G$107,"Women's Doubles",'Shuffled Matches'!$K$3:$K$107,"&lt;&gt;")=0,"",_xlfn.XLOOKUP(H21,$E$19:$E$24,$B$19:$B$24,""))</f>
-        <v>Team 6</v>
+        <v>Team 2</v>
       </c>
       <c r="J21" s="21">
         <f>IF(I21="","",_xlfn.XLOOKUP(H21,$E$19:$E$24,$C$19:$C$24,""))</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K21" s="53">
         <f>IF(I21="","",_xlfn.XLOOKUP(H21,$E$19:$E$24,$D$19:$D$24,""))</f>
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="L21" s="17">
         <f>'Points Table'!E28</f>
-        <v>82</v>
-      </c>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.15">
+        <v>75</v>
+      </c>
+      <c r="M21" s="59"/>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B22" s="19" t="s">
         <v>59</v>
       </c>
@@ -12462,7 +12466,7 @@
       </c>
       <c r="I22" s="22" t="str">
         <f>IF(COUNTIFS('Shuffled Matches'!$G$3:$G$107,"Women's Doubles",'Shuffled Matches'!$K$3:$K$107,"&lt;&gt;")=0,"",_xlfn.XLOOKUP(H22,$E$19:$E$24,$B$19:$B$24,""))</f>
-        <v>Team 2</v>
+        <v>Team 6</v>
       </c>
       <c r="J22" s="21">
         <f>IF(I22="","",_xlfn.XLOOKUP(H22,$E$19:$E$24,$C$19:$C$24,""))</f>
@@ -12470,14 +12474,14 @@
       </c>
       <c r="K22" s="53">
         <f>IF(I22="","",_xlfn.XLOOKUP(H22,$E$19:$E$24,$D$19:$D$24,""))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L22" s="17">
         <f>'Points Table'!E29</f>
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="23" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B23" s="19" t="s">
         <v>50</v>
       </c>
@@ -12507,7 +12511,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B24" s="19" t="s">
         <v>51</v>
       </c>
@@ -12521,7 +12525,7 @@
       </c>
       <c r="E24" s="20">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F24" s="17" t="str">
         <f>IF(COUNTIFS('Shuffled Matches'!$G$3:$G$107,"Women's Doubles",'Shuffled Matches'!$K$3:$K$107,"&lt;&gt;")=0,"Pending",IF(E24&lt;=4,"Top 4","Eliminated"))</f>
@@ -12537,7 +12541,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
@@ -12550,7 +12554,7 @@
       <c r="K25" s="17"/>
       <c r="L25" s="17"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -12563,7 +12567,7 @@
       <c r="K26" s="17"/>
       <c r="L26" s="17"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
@@ -12576,7 +12580,7 @@
       <c r="K27" s="17"/>
       <c r="L27" s="17"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="28" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
@@ -12589,7 +12593,7 @@
       <c r="K28" s="17"/>
       <c r="L28" s="17"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="29" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
@@ -12602,7 +12606,7 @@
       <c r="K29" s="17"/>
       <c r="L29" s="17"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="30" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B30" s="64" t="s">
         <v>141</v>
       </c>
@@ -12617,7 +12621,7 @@
       <c r="K30" s="64"/>
       <c r="L30" s="18"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="31" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B31" s="37" t="s">
         <v>241</v>
       </c>
@@ -12632,7 +12636,7 @@
       <c r="K31" s="37"/>
       <c r="L31" s="37"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.15">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.15">
       <c r="B32" s="16" t="s">
         <v>131</v>
       </c>
@@ -14703,15 +14707,15 @@
       </c>
       <c r="E10" s="13">
         <f>'Format Scoreboards'!C20</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F10" s="13">
         <f>'Format Scoreboards'!L20</f>
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G10" s="54">
         <f>'Format Scoreboards'!E20</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H10" s="13" t="str">
         <f t="shared" si="1"/>
@@ -14733,11 +14737,11 @@
       </c>
       <c r="E11" s="13">
         <f>'Format Scoreboards'!C21</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F11" s="13">
         <f>'Format Scoreboards'!L21</f>
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="G11" s="54">
         <f>'Format Scoreboards'!E21</f>
@@ -14831,7 +14835,7 @@
       </c>
       <c r="G14" s="54">
         <f>'Format Scoreboards'!E24</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" s="13" t="str">
         <f t="shared" si="1"/>
@@ -15789,26 +15793,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="66" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
     </row>
     <row r="2" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="67" t="s">
         <v>242</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A3" s="17"/>
@@ -16070,11 +16074,11 @@
       </c>
       <c r="B15" s="17" t="str">
         <f>INDEX('Qualification Data'!$D$9:$D$14,MATCH($A15,'Qualification Data'!$G$9:$G$14,0))</f>
-        <v>Neha P Jain + Drishti</v>
+        <v>Vaishnavi M + Keerthana</v>
       </c>
       <c r="C15" s="17" t="str">
         <f>INDEX('Qualification Data'!$C$9:$C$14,MATCH($A15,'Qualification Data'!$G$9:$G$14,0))</f>
-        <v>Team 6</v>
+        <v>Team 2</v>
       </c>
       <c r="D15" s="17" t="str">
         <f>INDEX('Qualification Data'!$B$9:$B$14,MATCH($A15,'Qualification Data'!$G$9:$G$14,0))</f>
@@ -16082,11 +16086,11 @@
       </c>
       <c r="E15" s="17">
         <f>INDEX('Qualification Data'!$E$9:$E$14,MATCH($A15,'Qualification Data'!$G$9:$G$14,0))</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F15" s="17">
         <f>INDEX('Qualification Data'!$F$9:$F$14,MATCH($A15,'Qualification Data'!$G$9:$G$14,0))</f>
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="G15" s="17" t="s">
         <v>156</v>
@@ -16098,11 +16102,11 @@
       </c>
       <c r="B16" s="17" t="str">
         <f>INDEX('Qualification Data'!$D$9:$D$14,MATCH($A16,'Qualification Data'!$G$9:$G$14,0))</f>
-        <v>Vaishnavi M + Keerthana</v>
+        <v>Neha P Jain + Drishti</v>
       </c>
       <c r="C16" s="17" t="str">
         <f>INDEX('Qualification Data'!$C$9:$C$14,MATCH($A16,'Qualification Data'!$G$9:$G$14,0))</f>
-        <v>Team 2</v>
+        <v>Team 6</v>
       </c>
       <c r="D16" s="17" t="str">
         <f>INDEX('Qualification Data'!$B$9:$B$14,MATCH($A16,'Qualification Data'!$G$9:$G$14,0))</f>
@@ -16114,7 +16118,7 @@
       </c>
       <c r="F16" s="17">
         <f>INDEX('Qualification Data'!$F$9:$F$14,MATCH($A16,'Qualification Data'!$G$9:$G$14,0))</f>
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="G16" s="17" t="s">
         <v>156</v>
@@ -16711,52 +16715,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.15">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="60" t="s">
         <v>174</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="60"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.15">
-      <c r="A2" s="68" t="s">
+      <c r="A2" s="61" t="s">
         <v>248</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="68"/>
-      <c r="R2" s="68"/>
-      <c r="S2" s="68"/>
-      <c r="T2" s="68"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="61"/>
+      <c r="L2" s="61"/>
+      <c r="M2" s="61"/>
+      <c r="N2" s="61"/>
+      <c r="O2" s="61"/>
+      <c r="P2" s="61"/>
+      <c r="Q2" s="61"/>
+      <c r="R2" s="61"/>
+      <c r="S2" s="61"/>
+      <c r="T2" s="61"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.15">
       <c r="A4" s="49" t="s">
@@ -16970,12 +16974,18 @@
         <f>IF(OR(R5="Pending",LEFT(R5,3)="Tie"),"TBD",R5)</f>
         <v>Team 6</v>
       </c>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29" t="str">
+      <c r="F7" s="29">
+        <v>21</v>
+      </c>
+      <c r="G7" s="29">
+        <v>21</v>
+      </c>
+      <c r="H7" s="29">
+        <v>0</v>
+      </c>
+      <c r="I7" s="29">
         <f t="shared" si="0"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="J7" s="30" t="s">
         <v>186</v>
@@ -16988,20 +16998,26 @@
         <f>IF(OR(R6="Pending",LEFT(R6,3)="Tie"),"TBD",R6)</f>
         <v>Team 4</v>
       </c>
-      <c r="M7" s="30"/>
-      <c r="N7" s="30"/>
-      <c r="O7" s="30"/>
-      <c r="P7" s="30" t="str">
+      <c r="M7" s="30">
+        <v>17</v>
+      </c>
+      <c r="N7" s="30">
+        <v>18</v>
+      </c>
+      <c r="O7" s="30">
+        <v>0</v>
+      </c>
+      <c r="P7" s="30">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q7" s="28" t="str">
         <f t="shared" si="2"/>
-        <v>Pending</v>
+        <v>Neha P Jain</v>
       </c>
       <c r="R7" s="28" t="str">
         <f t="shared" si="3"/>
-        <v>Pending</v>
+        <v>Team 6</v>
       </c>
       <c r="S7" s="30"/>
       <c r="T7" s="30"/>
@@ -17036,11 +17052,11 @@
       </c>
       <c r="K8" s="27" t="str">
         <f>Qualifiers!B16</f>
-        <v>Vaishnavi M + Keerthana</v>
+        <v>Neha P Jain + Drishti</v>
       </c>
       <c r="L8" s="27" t="str">
         <f>Qualifiers!C16</f>
-        <v>Team 2</v>
+        <v>Team 6</v>
       </c>
       <c r="M8" s="27"/>
       <c r="N8" s="27"/>
@@ -17078,38 +17094,50 @@
         <f>Qualifiers!C14</f>
         <v>Team 4</v>
       </c>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26" t="str">
+      <c r="F9" s="26">
+        <v>16</v>
+      </c>
+      <c r="G9" s="26">
+        <v>7</v>
+      </c>
+      <c r="H9" s="26">
+        <v>9</v>
+      </c>
+      <c r="I9" s="26">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1</v>
       </c>
       <c r="J9" s="27">
         <v>3</v>
       </c>
       <c r="K9" s="27" t="str">
         <f>Qualifiers!B15</f>
-        <v>Neha P Jain + Drishti</v>
+        <v>Vaishnavi M + Keerthana</v>
       </c>
       <c r="L9" s="27" t="str">
         <f>Qualifiers!C15</f>
-        <v>Team 6</v>
-      </c>
-      <c r="M9" s="27"/>
-      <c r="N9" s="27"/>
-      <c r="O9" s="27"/>
-      <c r="P9" s="27" t="str">
+        <v>Team 2</v>
+      </c>
+      <c r="M9" s="27">
+        <v>12</v>
+      </c>
+      <c r="N9" s="27">
+        <v>16</v>
+      </c>
+      <c r="O9" s="27">
+        <v>16</v>
+      </c>
+      <c r="P9" s="27">
         <f t="shared" si="1"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="Q9" s="25" t="str">
         <f t="shared" si="2"/>
-        <v>Pending</v>
+        <v>Vaishnavi M + Keerthana</v>
       </c>
       <c r="R9" s="25" t="str">
         <f t="shared" si="3"/>
-        <v>Pending</v>
+        <v>Team 2</v>
       </c>
       <c r="S9" s="27"/>
       <c r="T9" s="27"/>
@@ -17144,11 +17172,11 @@
       </c>
       <c r="K10" s="30" t="str">
         <f>IF(OR(Q9="Pending",LEFT(Q9,3)="Tie"),"TBD",Q9)</f>
-        <v>TBD</v>
+        <v>Vaishnavi M + Keerthana</v>
       </c>
       <c r="L10" s="30" t="str">
         <f>IF(OR(R9="Pending",LEFT(R9,3)="Tie"),"TBD",R9)</f>
-        <v>TBD</v>
+        <v>Team 2</v>
       </c>
       <c r="M10" s="30"/>
       <c r="N10" s="30"/>
@@ -17504,12 +17532,18 @@
         <f>Qualifiers!D29</f>
         <v>Team 1</v>
       </c>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="32"/>
-      <c r="I16" s="32" t="str">
+      <c r="F16" s="32">
+        <v>9</v>
+      </c>
+      <c r="G16" s="32">
+        <v>14</v>
+      </c>
+      <c r="H16" s="32">
+        <v>0</v>
+      </c>
+      <c r="I16" s="32">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J16" s="33" t="s">
         <v>192</v>
@@ -17522,28 +17556,34 @@
         <f>Qualifiers!G29</f>
         <v>Team 5</v>
       </c>
-      <c r="M16" s="33"/>
-      <c r="N16" s="33"/>
-      <c r="O16" s="33"/>
-      <c r="P16" s="33" t="str">
+      <c r="M16" s="33">
+        <v>16</v>
+      </c>
+      <c r="N16" s="33">
+        <v>16</v>
+      </c>
+      <c r="O16" s="33">
+        <v>0</v>
+      </c>
+      <c r="P16" s="33">
         <f t="shared" si="1"/>
-        <v/>
+        <v>2</v>
       </c>
       <c r="Q16" s="31" t="str">
         <f>IF(MAX(N(I16),N(P16))&gt;=2,IF(I16&gt;P16,D16,K16),IF(AND(COUNT(F16:H16,M16:O16)=6,I16=P16),"Tie - review","Pending"))</f>
-        <v>Pending</v>
+        <v>Vidwan</v>
       </c>
       <c r="R16" s="31" t="str">
         <f>IF(OR(Q16="Pending",LEFT(Q16,3)="Tie"),Q16,IF(Q16=D16,E16,L16))</f>
-        <v>Pending</v>
-      </c>
-      <c r="S16" s="33" t="str">
+        <v>Team 5</v>
+      </c>
+      <c r="S16" s="33">
         <f>IF(OR(Q16="Pending",LEFT(Q16,3)="Tie"),"",SUMIF('Qualification Data'!$D$23:$D$34,Q16,'Qualification Data'!$F$23:$F$34)+IF(Q16=D16,SUM(F16:H16),SUM(M16:O16)))</f>
-        <v/>
-      </c>
-      <c r="T16" s="33" t="str">
+        <v>129</v>
+      </c>
+      <c r="T16" s="33">
         <f>IF(S16="","",1+COUNTIF($S$14:$S$17,"&gt;"&amp;S16)+COUNTIF($S$14:S16,S16)-1)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.15">
@@ -17638,11 +17678,11 @@
       </c>
       <c r="K18" s="27" t="str">
         <f>IF(OR(Q16="Pending",LEFT(Q16,3)="Tie",Q16=""),"TBD",Q16)</f>
-        <v>TBD</v>
+        <v>Vidwan</v>
       </c>
       <c r="L18" s="27" t="str">
         <f>IF(K18="TBD","TBD",R16)</f>
-        <v>TBD</v>
+        <v>Team 5</v>
       </c>
       <c r="M18" s="27"/>
       <c r="N18" s="27"/>
@@ -18248,32 +18288,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="66" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
     </row>
     <row r="2" spans="1:10" ht="34" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="60" t="s">
+      <c r="A2" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="I2" s="60"/>
-      <c r="J2" s="60"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A3" s="17"/>
@@ -18366,15 +18406,15 @@
       </c>
       <c r="B6" s="35">
         <f>COUNTIF('Shuffled Matches'!$L$3:$L$112,$A6)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="35">
         <f>SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A6,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A6,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A6,Finals!$B$5:$B$28,"Semifinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A6,Finals!$B$5:$B$28,"Semifinal*")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D6" s="35">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E6" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A6,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
@@ -18394,11 +18434,11 @@
       </c>
       <c r="I6" s="36">
         <f t="shared" ref="I6:I10" si="3">D6+G6+H6</f>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="J6" s="36">
         <f t="shared" ref="J6:J10" si="4">_xlfn.RANK.EQ(I6,$I$5:$I$10,0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.15">
@@ -18407,7 +18447,7 @@
       </c>
       <c r="B7" s="35">
         <f>COUNTIF('Shuffled Matches'!$L$3:$L$112,$A7)</f>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" s="35">
         <f>SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A7,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A7,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A7,Finals!$B$5:$B$28,"Semifinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A7,Finals!$B$5:$B$28,"Semifinal*")</f>
@@ -18415,7 +18455,7 @@
       </c>
       <c r="D7" s="35">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A7,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
@@ -18435,11 +18475,11 @@
       </c>
       <c r="I7" s="36">
         <f t="shared" si="3"/>
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J7" s="36">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="48" customFormat="1" x14ac:dyDescent="0.15">
@@ -18452,11 +18492,11 @@
       </c>
       <c r="C8" s="35">
         <f>SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A8,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A8,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A8,Finals!$B$5:$B$28,"Semifinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A8,Finals!$B$5:$B$28,"Semifinal*")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="35">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A8,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
@@ -18464,7 +18504,7 @@
       </c>
       <c r="F8" s="35" cm="1">
         <f t="array" ref="F8">SUMPRODUCT((Finals!$B$5:$B$28="Final")*(LEFT(Finals!$R$5:$R$28,4)="Team")*(Finals!$R$5:$R$28&lt;&gt;$A8)*(LEFT(Finals!$E$5:$E$28,4)="Team")*(LEFT(Finals!$L$5:$L$28,4)="Team")*--(((Finals!$E$5:$E$28=$A8)+(Finals!$L$5:$L$28=$A8))&gt;0)*--(Finals!$E$5:$E$28&lt;&gt;Finals!$L$5:$L$28))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="35">
         <f t="shared" si="1"/>
@@ -18472,11 +18512,11 @@
       </c>
       <c r="H8" s="35">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I8" s="36">
         <f t="shared" si="3"/>
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="J8" s="36">
         <f t="shared" si="4"/>
@@ -18493,11 +18533,11 @@
       </c>
       <c r="C9" s="35">
         <f>SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A9,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A9,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A9,Finals!$B$5:$B$28,"Semifinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A9,Finals!$B$5:$B$28,"Semifinal*")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="35">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E9" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A9,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
@@ -18517,7 +18557,7 @@
       </c>
       <c r="I9" s="36">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J9" s="36">
         <f t="shared" si="4"/>
@@ -18542,7 +18582,7 @@
       </c>
       <c r="E10" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A10,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="35" cm="1">
         <f t="array" ref="F10">SUMPRODUCT((Finals!$B$5:$B$28="Final")*(LEFT(Finals!$R$5:$R$28,4)="Team")*(Finals!$R$5:$R$28&lt;&gt;$A10)*(LEFT(Finals!$E$5:$E$28,4)="Team")*(LEFT(Finals!$L$5:$L$28,4)="Team")*--(((Finals!$E$5:$E$28=$A10)+(Finals!$L$5:$L$28=$A10))&gt;0)*--(Finals!$E$5:$E$28&lt;&gt;Finals!$L$5:$L$28))</f>
@@ -18550,7 +18590,7 @@
       </c>
       <c r="G10" s="35">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H10" s="35">
         <f t="shared" si="2"/>
@@ -18558,7 +18598,7 @@
       </c>
       <c r="I10" s="36">
         <f t="shared" si="3"/>
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="J10" s="36">
         <f t="shared" si="4"/>
@@ -18566,18 +18606,18 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="69" t="s">
         <v>210</v>
       </c>
-      <c r="B11" s="61"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61"/>
-      <c r="F11" s="61"/>
-      <c r="G11" s="61"/>
-      <c r="H11" s="61"/>
-      <c r="I11" s="61"/>
-      <c r="J11" s="61"/>
+      <c r="B11" s="69"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -18600,40 +18640,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="71" t="s">
         <v>230</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="72" t="s">
         <v>231</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="70" t="s">
         <v>232</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
-      <c r="D4" s="69"/>
-      <c r="E4" s="69"/>
-      <c r="F4" s="69"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="69"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="70"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="50" t="s">
@@ -18700,27 +18740,27 @@
       </c>
       <c r="B7">
         <f>COUNTIFS('Shuffled Matches'!$L$3:$L$107,$A7)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C7">
         <f>COUNTIFS('Shuffled Matches'!$D$3:$D$107,$A7,'Shuffled Matches'!$L$3:$L$107,"Team*")+COUNTIFS('Shuffled Matches'!$E$3:$E$107,$A7,'Shuffled Matches'!$L$3:$L$107,"Team*")-B7</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D7" s="50">
         <f t="shared" si="0"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E7">
         <f>SUMIFS('Shuffled Matches'!$N$3:$N$107,'Shuffled Matches'!$D$3:$D$107,$A7)+SUMIFS('Shuffled Matches'!$O$3:$O$107,'Shuffled Matches'!$E$3:$E$107,$A7)</f>
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="F7">
         <f>SUMIFS('Shuffled Matches'!$O$3:$O$107,'Shuffled Matches'!$D$3:$D$107,$A7)+SUMIFS('Shuffled Matches'!$N$3:$N$107,'Shuffled Matches'!$E$3:$E$107,$A7)</f>
-        <v>579</v>
+        <v>572</v>
       </c>
       <c r="G7" s="51">
         <f t="shared" si="1"/>
-        <v>-47</v>
+        <v>-33</v>
       </c>
       <c r="H7">
         <f t="shared" si="2"/>
@@ -18733,27 +18773,27 @@
       </c>
       <c r="B8">
         <f>COUNTIFS('Shuffled Matches'!$L$3:$L$107,$A8)</f>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C8">
         <f>COUNTIFS('Shuffled Matches'!$D$3:$D$107,$A8,'Shuffled Matches'!$L$3:$L$107,"Team*")+COUNTIFS('Shuffled Matches'!$E$3:$E$107,$A8,'Shuffled Matches'!$L$3:$L$107,"Team*")-B8</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" s="50">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E8">
         <f>SUMIFS('Shuffled Matches'!$N$3:$N$107,'Shuffled Matches'!$D$3:$D$107,$A8)+SUMIFS('Shuffled Matches'!$O$3:$O$107,'Shuffled Matches'!$E$3:$E$107,$A8)</f>
-        <v>650</v>
+        <v>643</v>
       </c>
       <c r="F8">
         <f>SUMIFS('Shuffled Matches'!$O$3:$O$107,'Shuffled Matches'!$D$3:$D$107,$A8)+SUMIFS('Shuffled Matches'!$N$3:$N$107,'Shuffled Matches'!$E$3:$E$107,$A8)</f>
-        <v>615</v>
+        <v>622</v>
       </c>
       <c r="G8" s="51">
         <f t="shared" si="1"/>
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
@@ -18860,16 +18900,16 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="69" t="s">
+      <c r="A14" s="70" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="69"/>
-      <c r="C14" s="69"/>
-      <c r="D14" s="69"/>
-      <c r="E14" s="69"/>
-      <c r="F14" s="69"/>
-      <c r="G14" s="69"/>
-      <c r="H14" s="69"/>
+      <c r="B14" s="70"/>
+      <c r="C14" s="70"/>
+      <c r="D14" s="70"/>
+      <c r="E14" s="70"/>
+      <c r="F14" s="70"/>
+      <c r="G14" s="70"/>
+      <c r="H14" s="70"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="50" t="s">
@@ -19096,16 +19136,16 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="69" t="s">
+      <c r="A24" s="70" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="69"/>
-      <c r="C24" s="69"/>
-      <c r="D24" s="69"/>
-      <c r="E24" s="69"/>
-      <c r="F24" s="69"/>
-      <c r="G24" s="69"/>
-      <c r="H24" s="69"/>
+      <c r="B24" s="70"/>
+      <c r="C24" s="70"/>
+      <c r="D24" s="70"/>
+      <c r="E24" s="70"/>
+      <c r="F24" s="70"/>
+      <c r="G24" s="70"/>
+      <c r="H24" s="70"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="50" t="s">
@@ -19172,31 +19212,31 @@
       </c>
       <c r="B27">
         <f>COUNTIFS('Shuffled Matches'!$L$3:$L$107,$A27,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27">
         <f>COUNTIFS('Shuffled Matches'!$D$3:$D$107,$A27,'Shuffled Matches'!$L$3:$L$107,"Team*",'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")+COUNTIFS('Shuffled Matches'!$E$3:$E$107,$A27,'Shuffled Matches'!$L$3:$L$107,"Team*",'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")-B27</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="50">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E27">
         <f>SUMIFS('Shuffled Matches'!$N$3:$N$107,'Shuffled Matches'!$D$3:$D$107,$A27,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")+SUMIFS('Shuffled Matches'!$O$3:$O$107,'Shuffled Matches'!$E$3:$E$107,$A27,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")</f>
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F27">
         <f>SUMIFS('Shuffled Matches'!$O$3:$O$107,'Shuffled Matches'!$D$3:$D$107,$A27,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")+SUMIFS('Shuffled Matches'!$N$3:$N$107,'Shuffled Matches'!$E$3:$E$107,$A27,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")</f>
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="G27" s="51">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="H27">
         <f t="shared" si="8"/>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
@@ -19205,27 +19245,27 @@
       </c>
       <c r="B28">
         <f>COUNTIFS('Shuffled Matches'!$L$3:$L$107,$A28,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C28">
         <f>COUNTIFS('Shuffled Matches'!$D$3:$D$107,$A28,'Shuffled Matches'!$L$3:$L$107,"Team*",'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")+COUNTIFS('Shuffled Matches'!$E$3:$E$107,$A28,'Shuffled Matches'!$L$3:$L$107,"Team*",'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")-B28</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D28" s="50">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E28">
         <f>SUMIFS('Shuffled Matches'!$N$3:$N$107,'Shuffled Matches'!$D$3:$D$107,$A28,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")+SUMIFS('Shuffled Matches'!$O$3:$O$107,'Shuffled Matches'!$E$3:$E$107,$A28,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")</f>
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="F28">
         <f>SUMIFS('Shuffled Matches'!$O$3:$O$107,'Shuffled Matches'!$D$3:$D$107,$A28,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")+SUMIFS('Shuffled Matches'!$N$3:$N$107,'Shuffled Matches'!$E$3:$E$107,$A28,'Shuffled Matches'!$G$3:$G$107,"Women's Doubles")</f>
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="G28" s="51">
         <f t="shared" si="7"/>
-        <v>-10</v>
+        <v>-24</v>
       </c>
       <c r="H28">
         <f t="shared" si="8"/>
@@ -19328,20 +19368,20 @@
       </c>
       <c r="H31">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="69" t="s">
+      <c r="A34" s="70" t="s">
         <v>17</v>
       </c>
-      <c r="B34" s="69"/>
-      <c r="C34" s="69"/>
-      <c r="D34" s="69"/>
-      <c r="E34" s="69"/>
-      <c r="F34" s="69"/>
-      <c r="G34" s="69"/>
-      <c r="H34" s="69"/>
+      <c r="B34" s="70"/>
+      <c r="C34" s="70"/>
+      <c r="D34" s="70"/>
+      <c r="E34" s="70"/>
+      <c r="F34" s="70"/>
+      <c r="G34" s="70"/>
+      <c r="H34" s="70"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="50" t="s">
@@ -19568,16 +19608,16 @@
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" s="69" t="s">
+      <c r="A44" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="B44" s="69"/>
-      <c r="C44" s="69"/>
-      <c r="D44" s="69"/>
-      <c r="E44" s="69"/>
-      <c r="F44" s="69"/>
-      <c r="G44" s="69"/>
-      <c r="H44" s="69"/>
+      <c r="B44" s="70"/>
+      <c r="C44" s="70"/>
+      <c r="D44" s="70"/>
+      <c r="E44" s="70"/>
+      <c r="F44" s="70"/>
+      <c r="G44" s="70"/>
+      <c r="H44" s="70"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="50" t="s">
@@ -19804,16 +19844,16 @@
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A54" s="69" t="s">
+      <c r="A54" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="B54" s="69"/>
-      <c r="C54" s="69"/>
-      <c r="D54" s="69"/>
-      <c r="E54" s="69"/>
-      <c r="F54" s="69"/>
-      <c r="G54" s="69"/>
-      <c r="H54" s="69"/>
+      <c r="B54" s="70"/>
+      <c r="C54" s="70"/>
+      <c r="D54" s="70"/>
+      <c r="E54" s="70"/>
+      <c r="F54" s="70"/>
+      <c r="G54" s="70"/>
+      <c r="H54" s="70"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="50" t="s">
@@ -20040,16 +20080,16 @@
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A64" s="69" t="s">
+      <c r="A64" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="B64" s="69"/>
-      <c r="C64" s="69"/>
-      <c r="D64" s="69"/>
-      <c r="E64" s="69"/>
-      <c r="F64" s="69"/>
-      <c r="G64" s="69"/>
-      <c r="H64" s="69"/>
+      <c r="B64" s="70"/>
+      <c r="C64" s="70"/>
+      <c r="D64" s="70"/>
+      <c r="E64" s="70"/>
+      <c r="F64" s="70"/>
+      <c r="G64" s="70"/>
+      <c r="H64" s="70"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="50" t="s">
@@ -20276,16 +20316,16 @@
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A74" s="69" t="s">
+      <c r="A74" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="B74" s="69"/>
-      <c r="C74" s="69"/>
-      <c r="D74" s="69"/>
-      <c r="E74" s="69"/>
-      <c r="F74" s="69"/>
-      <c r="G74" s="69"/>
-      <c r="H74" s="69"/>
+      <c r="B74" s="70"/>
+      <c r="C74" s="70"/>
+      <c r="D74" s="70"/>
+      <c r="E74" s="70"/>
+      <c r="F74" s="70"/>
+      <c r="G74" s="70"/>
+      <c r="H74" s="70"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="50" t="s">

</xml_diff>

<commit_message>
Scores from Score_Card_6: MS QF2-QF4 and SF2, MD QF2; knockout teams checked against the roster
Jay B (Team 4) into the Men's Singles final; Kunal D + Anirudha H (Team 3)
win MD QF2; Team 3 lead Best Team on 34. Points match the Excel, including
the 1-0 third-set entries. The Finals sheet's team formulas had Sujal as
Team 5 and Vidwan as Team 3 in the semifinals; competitors now keep their
group-stage team (converter and live sheet reader).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KpjSian9KihxBdn7Md9Nh1
</commit_message>
<xml_diff>
--- a/scores/Score_Card.xlsx
+++ b/scores/Score_Card.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliakber/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliakber/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A03DEF97-D341-7948-99A5-F5175C407AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{02480FB2-6F29-FB40-8734-4001B081B5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16960" activeTab="6" xr2:uid="{80F890F9-808C-4260-AFEB-091B93DC4636}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{80F890F9-808C-4260-AFEB-091B93DC4636}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -1119,7 +1119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1283,19 +1283,13 @@
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1306,6 +1300,12 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1315,6 +1315,9 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6310,7 +6313,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="9" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B9" s="41" t="s">
         <v>10</v>
       </c>
@@ -6609,7 +6612,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="15" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B15" s="41" t="s">
         <v>10</v>
       </c>
@@ -6659,7 +6662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="16" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B16" s="41" t="s">
         <v>10</v>
       </c>
@@ -6959,7 +6962,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.15">
       <c r="B22" s="41" t="s">
         <v>26</v>
       </c>
@@ -8059,7 +8062,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="44" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B44" s="41" t="s">
         <v>31</v>
       </c>
@@ -8409,7 +8412,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B51" s="41" t="s">
         <v>34</v>
       </c>
@@ -8809,7 +8812,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B59" s="41" t="s">
         <v>37</v>
       </c>
@@ -9109,7 +9112,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="65" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B65" s="41" t="s">
         <v>37</v>
       </c>
@@ -9409,7 +9412,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="71" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B71" s="41" t="s">
         <v>37</v>
       </c>
@@ -9509,7 +9512,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="73" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B73" s="41" t="s">
         <v>40</v>
       </c>
@@ -9759,7 +9762,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="78" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="78" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B78" s="41" t="s">
         <v>40</v>
       </c>
@@ -9959,7 +9962,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="82" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B82" s="41" t="s">
         <v>40</v>
       </c>
@@ -10309,7 +10312,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="89" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B89" s="41" t="s">
         <v>43</v>
       </c>
@@ -10810,7 +10813,7 @@
         <v>-15</v>
       </c>
     </row>
-    <row r="99" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="99" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B99" s="41" t="s">
         <v>43</v>
       </c>
@@ -11109,7 +11112,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="2:16" x14ac:dyDescent="0.15">
+    <row r="105" spans="2:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="B105" s="41" t="s">
         <v>46</v>
       </c>
@@ -11276,10 +11279,8 @@
     </row>
   </sheetData>
   <autoFilter ref="B2:M107" xr:uid="{8D08637B-F719-49C8-8CD0-A0482E45DECD}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="Women's Doubles"/>
-      </filters>
+    <filterColumn colId="10">
+      <filters blank="1"/>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="J3:K92 K93 J94:K102 J103:J107 K103:K112">
@@ -11316,36 +11317,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="24" x14ac:dyDescent="0.2">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="61" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
     </row>
     <row r="2" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="62" t="s">
         <v>240</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
-      <c r="I2" s="63"/>
-      <c r="J2" s="63"/>
-      <c r="K2" s="63"/>
-      <c r="L2" s="63"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
     </row>
     <row r="3" spans="1:12" ht="18" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -11902,18 +11903,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="60" t="s">
         <v>137</v>
       </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="I2" s="60"/>
+      <c r="J2" s="60"/>
+      <c r="K2" s="60"/>
       <c r="L2" s="18"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.15">
@@ -12254,18 +12255,18 @@
       <c r="L15" s="17"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B16" s="64" t="s">
+      <c r="B16" s="60" t="s">
         <v>140</v>
       </c>
-      <c r="C16" s="64"/>
-      <c r="D16" s="64"/>
-      <c r="E16" s="64"/>
-      <c r="F16" s="64"/>
-      <c r="G16" s="64"/>
-      <c r="H16" s="64"/>
-      <c r="I16" s="64"/>
-      <c r="J16" s="64"/>
-      <c r="K16" s="64"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="60"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="60"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="60"/>
+      <c r="I16" s="60"/>
+      <c r="J16" s="60"/>
+      <c r="K16" s="60"/>
       <c r="L16" s="18"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.15">
@@ -12607,18 +12608,18 @@
       <c r="L29" s="17"/>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.15">
-      <c r="B30" s="64" t="s">
+      <c r="B30" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="C30" s="64"/>
-      <c r="D30" s="64"/>
-      <c r="E30" s="64"/>
-      <c r="F30" s="64"/>
-      <c r="G30" s="64"/>
-      <c r="H30" s="64"/>
-      <c r="I30" s="64"/>
-      <c r="J30" s="64"/>
-      <c r="K30" s="64"/>
+      <c r="C30" s="60"/>
+      <c r="D30" s="60"/>
+      <c r="E30" s="60"/>
+      <c r="F30" s="60"/>
+      <c r="G30" s="60"/>
+      <c r="H30" s="60"/>
+      <c r="I30" s="60"/>
+      <c r="J30" s="60"/>
+      <c r="K30" s="60"/>
       <c r="L30" s="18"/>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.15">
@@ -12959,18 +12960,18 @@
       <c r="L43" s="17"/>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B44" s="64" t="s">
+      <c r="B44" s="60" t="s">
         <v>142</v>
       </c>
-      <c r="C44" s="64"/>
-      <c r="D44" s="64"/>
-      <c r="E44" s="64"/>
-      <c r="F44" s="64"/>
-      <c r="G44" s="64"/>
-      <c r="H44" s="64"/>
-      <c r="I44" s="64"/>
-      <c r="J44" s="64"/>
-      <c r="K44" s="64"/>
+      <c r="C44" s="60"/>
+      <c r="D44" s="60"/>
+      <c r="E44" s="60"/>
+      <c r="F44" s="60"/>
+      <c r="G44" s="60"/>
+      <c r="H44" s="60"/>
+      <c r="I44" s="60"/>
+      <c r="J44" s="60"/>
+      <c r="K44" s="60"/>
       <c r="L44" s="18"/>
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.15">
@@ -13311,18 +13312,18 @@
       <c r="L57" s="17"/>
     </row>
     <row r="58" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B58" s="64" t="s">
+      <c r="B58" s="60" t="s">
         <v>143</v>
       </c>
-      <c r="C58" s="64"/>
-      <c r="D58" s="64"/>
-      <c r="E58" s="64"/>
-      <c r="F58" s="64"/>
-      <c r="G58" s="64"/>
-      <c r="H58" s="64"/>
-      <c r="I58" s="64"/>
-      <c r="J58" s="64"/>
-      <c r="K58" s="64"/>
+      <c r="C58" s="60"/>
+      <c r="D58" s="60"/>
+      <c r="E58" s="60"/>
+      <c r="F58" s="60"/>
+      <c r="G58" s="60"/>
+      <c r="H58" s="60"/>
+      <c r="I58" s="60"/>
+      <c r="J58" s="60"/>
+      <c r="K58" s="60"/>
       <c r="L58" s="18"/>
     </row>
     <row r="59" spans="2:12" x14ac:dyDescent="0.15">
@@ -13663,18 +13664,18 @@
       <c r="L71" s="17"/>
     </row>
     <row r="72" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B72" s="64" t="s">
+      <c r="B72" s="60" t="s">
         <v>144</v>
       </c>
-      <c r="C72" s="64"/>
-      <c r="D72" s="64"/>
-      <c r="E72" s="64"/>
-      <c r="F72" s="64"/>
-      <c r="G72" s="64"/>
-      <c r="H72" s="64"/>
-      <c r="I72" s="64"/>
-      <c r="J72" s="64"/>
-      <c r="K72" s="64"/>
+      <c r="C72" s="60"/>
+      <c r="D72" s="60"/>
+      <c r="E72" s="60"/>
+      <c r="F72" s="60"/>
+      <c r="G72" s="60"/>
+      <c r="H72" s="60"/>
+      <c r="I72" s="60"/>
+      <c r="J72" s="60"/>
+      <c r="K72" s="60"/>
       <c r="L72" s="18"/>
     </row>
     <row r="73" spans="2:12" x14ac:dyDescent="0.15">
@@ -14015,18 +14016,18 @@
       <c r="L85" s="17"/>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.15">
-      <c r="B86" s="64" t="s">
+      <c r="B86" s="60" t="s">
         <v>145</v>
       </c>
-      <c r="C86" s="64"/>
-      <c r="D86" s="64"/>
-      <c r="E86" s="64"/>
-      <c r="F86" s="64"/>
-      <c r="G86" s="64"/>
-      <c r="H86" s="64"/>
-      <c r="I86" s="64"/>
-      <c r="J86" s="64"/>
-      <c r="K86" s="64"/>
+      <c r="C86" s="60"/>
+      <c r="D86" s="60"/>
+      <c r="E86" s="60"/>
+      <c r="F86" s="60"/>
+      <c r="G86" s="60"/>
+      <c r="H86" s="60"/>
+      <c r="I86" s="60"/>
+      <c r="J86" s="60"/>
+      <c r="K86" s="60"/>
       <c r="L86" s="18"/>
     </row>
     <row r="87" spans="2:12" x14ac:dyDescent="0.15">
@@ -15779,7 +15780,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E626B811-43F6-40AF-9C49-487E0D1B9ADB}">
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="11.83203125" style="14" bestFit="1" customWidth="1"/>
@@ -15793,26 +15794,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="64" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
     </row>
     <row r="2" spans="1:7" ht="29.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="65" t="s">
         <v>242</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A3" s="17"/>
@@ -15824,15 +15825,15 @@
       <c r="G3" s="17"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="63" t="s">
         <v>154</v>
       </c>
-      <c r="B4" s="65"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A5" s="23" t="s">
@@ -15979,15 +15980,15 @@
       <c r="G10" s="17"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="63" t="s">
         <v>157</v>
       </c>
-      <c r="B11" s="65"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65"/>
-      <c r="G11" s="65"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A12" s="23" t="s">
@@ -16134,15 +16135,15 @@
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A18" s="65" t="s">
+      <c r="A18" s="63" t="s">
         <v>158</v>
       </c>
-      <c r="B18" s="65"/>
-      <c r="C18" s="65"/>
-      <c r="D18" s="65"/>
-      <c r="E18" s="65"/>
-      <c r="F18" s="65"/>
-      <c r="G18" s="65"/>
+      <c r="B18" s="63"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A19" s="23" t="s">
@@ -16289,15 +16290,15 @@
       <c r="G24" s="17"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A25" s="65" t="s">
+      <c r="A25" s="63" t="s">
         <v>159</v>
       </c>
-      <c r="B25" s="65"/>
-      <c r="C25" s="65"/>
-      <c r="D25" s="65"/>
-      <c r="E25" s="65"/>
-      <c r="F25" s="65"/>
-      <c r="G25" s="65"/>
+      <c r="B25" s="63"/>
+      <c r="C25" s="63"/>
+      <c r="D25" s="63"/>
+      <c r="E25" s="63"/>
+      <c r="F25" s="63"/>
+      <c r="G25" s="63"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A26" s="23" t="s">
@@ -16437,252 +16438,171 @@
       <c r="D31" s="17"/>
       <c r="E31" s="17"/>
       <c r="F31" s="17"/>
-      <c r="G31" s="24"/>
+      <c r="G31" s="73"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A32" s="17"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="24"/>
+      <c r="A32" s="63" t="s">
+        <v>169</v>
+      </c>
+      <c r="B32" s="63"/>
+      <c r="C32" s="63"/>
+      <c r="D32" s="63"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="63"/>
+      <c r="G32" s="63"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A33" s="17"/>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="24"/>
+      <c r="A33" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="B33" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="F33" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="G33" s="23" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A34" s="17"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="24"/>
+      <c r="A34" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="B34" s="17">
+        <v>1</v>
+      </c>
+      <c r="C34" s="17" t="str" cm="1">
+        <f t="array" ref="C34">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B34,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
+        <v>Kushal + Shubham</v>
+      </c>
+      <c r="D34" s="17" t="str" cm="1">
+        <f t="array" ref="D34">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B34,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
+        <v>Team 2</v>
+      </c>
+      <c r="E34" s="17">
+        <v>4</v>
+      </c>
+      <c r="F34" s="17" t="str" cm="1">
+        <f t="array" ref="F34">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E34,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
+        <v>Khush B + Hemanth</v>
+      </c>
+      <c r="G34" s="24" t="str" cm="1">
+        <f t="array" ref="G34">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E34,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
+        <v>Team 4</v>
+      </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A35" s="17"/>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
+      <c r="A35" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="B35" s="17">
+        <v>2</v>
+      </c>
+      <c r="C35" s="17" t="str" cm="1">
+        <f t="array" ref="C35">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B35,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
+        <v>Kunal D + Anirudha H</v>
+      </c>
+      <c r="D35" s="17" t="str" cm="1">
+        <f t="array" ref="D35">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B35,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
+        <v>Team 3</v>
+      </c>
+      <c r="E35" s="17">
+        <v>3</v>
+      </c>
+      <c r="F35" s="17" t="str" cm="1">
+        <f t="array" ref="F35">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E35,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
+        <v>Yuvraj + Karthik KB</v>
+      </c>
+      <c r="G35" s="24" t="str" cm="1">
+        <f t="array" ref="G35">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E35,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
+        <v>Team 2</v>
+      </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A36" s="17"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="17"/>
+      <c r="A36" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="B36" s="17">
+        <v>3</v>
+      </c>
+      <c r="C36" s="17" t="str" cm="1">
+        <f t="array" ref="C36">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B36,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
+        <v>Leela Sagar + Ali Akbar</v>
+      </c>
+      <c r="D36" s="17" t="str" cm="1">
+        <f t="array" ref="D36">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B36,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
+        <v>Team 4</v>
+      </c>
+      <c r="E36" s="17">
+        <v>2</v>
+      </c>
+      <c r="F36" s="17" t="str" cm="1">
+        <f t="array" ref="F36">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E36,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
+        <v>Sarvesh H + Deviprasad</v>
+      </c>
+      <c r="G36" s="24" t="str" cm="1">
+        <f t="array" ref="G36">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E36,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
+        <v>Team 3</v>
+      </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A37" s="17"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="17"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="17"/>
-      <c r="F37" s="17"/>
-      <c r="G37" s="17"/>
+      <c r="A37" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="B37" s="17">
+        <v>4</v>
+      </c>
+      <c r="C37" s="17" t="str" cm="1">
+        <f t="array" ref="C37">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B37,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
+        <v>Nagarajan + Chandrashaker Joshi</v>
+      </c>
+      <c r="D37" s="17" t="str" cm="1">
+        <f t="array" ref="D37">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B37,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
+        <v>Team 6</v>
+      </c>
+      <c r="E37" s="17">
+        <v>1</v>
+      </c>
+      <c r="F37" s="17" t="str" cm="1">
+        <f t="array" ref="F37">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E37,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
+        <v>Rohan + Bhuvanesh</v>
+      </c>
+      <c r="G37" s="24" t="str" cm="1">
+        <f t="array" ref="G37">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E37,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
+        <v>Team 6</v>
+      </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A38" s="65" t="s">
-        <v>169</v>
-      </c>
-      <c r="B38" s="65"/>
-      <c r="C38" s="65"/>
-      <c r="D38" s="65"/>
-      <c r="E38" s="65"/>
-      <c r="F38" s="65"/>
-      <c r="G38" s="65"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A39" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="B39" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="C39" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="D39" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="E39" s="23" t="s">
-        <v>172</v>
-      </c>
-      <c r="F39" s="23" t="s">
-        <v>173</v>
-      </c>
-      <c r="G39" s="23" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A40" s="17" t="s">
-        <v>165</v>
-      </c>
-      <c r="B40" s="17">
-        <v>1</v>
-      </c>
-      <c r="C40" s="17" t="str" cm="1">
-        <f t="array" ref="C40">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B40,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
-        <v>Kushal + Shubham</v>
-      </c>
-      <c r="D40" s="17" t="str" cm="1">
-        <f t="array" ref="D40">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B40,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
-        <v>Team 2</v>
-      </c>
-      <c r="E40" s="17">
-        <v>4</v>
-      </c>
-      <c r="F40" s="17" t="str" cm="1">
-        <f t="array" ref="F40">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E40,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
-        <v>Khush B + Hemanth</v>
-      </c>
-      <c r="G40" s="24" t="str" cm="1">
-        <f t="array" ref="G40">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E40,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
-        <v>Team 4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A41" s="17" t="s">
-        <v>166</v>
-      </c>
-      <c r="B41" s="17">
-        <v>2</v>
-      </c>
-      <c r="C41" s="17" t="str" cm="1">
-        <f t="array" ref="C41">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B41,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
-        <v>Kunal D + Anirudha H</v>
-      </c>
-      <c r="D41" s="17" t="str" cm="1">
-        <f t="array" ref="D41">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B41,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
-        <v>Team 3</v>
-      </c>
-      <c r="E41" s="17">
-        <v>3</v>
-      </c>
-      <c r="F41" s="17" t="str" cm="1">
-        <f t="array" ref="F41">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E41,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
-        <v>Yuvraj + Karthik KB</v>
-      </c>
-      <c r="G41" s="24" t="str" cm="1">
-        <f t="array" ref="G41">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E41,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
-        <v>Team 2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A42" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="B42" s="17">
-        <v>3</v>
-      </c>
-      <c r="C42" s="17" t="str" cm="1">
-        <f t="array" ref="C42">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B42,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
-        <v>Leela Sagar + Ali Akbar</v>
-      </c>
-      <c r="D42" s="17" t="str" cm="1">
-        <f t="array" ref="D42">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B42,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
-        <v>Team 4</v>
-      </c>
-      <c r="E42" s="17">
-        <v>2</v>
-      </c>
-      <c r="F42" s="17" t="str" cm="1">
-        <f t="array" ref="F42">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E42,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
-        <v>Sarvesh H + Deviprasad</v>
-      </c>
-      <c r="G42" s="24" t="str" cm="1">
-        <f t="array" ref="G42">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E42,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
-        <v>Team 3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A43" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="B43" s="17">
-        <v>4</v>
-      </c>
-      <c r="C43" s="17" t="str" cm="1">
-        <f t="array" ref="C43">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B43,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
-        <v>Nagarajan + Chandrashaker Joshi</v>
-      </c>
-      <c r="D43" s="17" t="str" cm="1">
-        <f t="array" ref="D43">_xlfn.XLOOKUP("Men's Doubles 1"&amp;B43,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
-        <v>Team 6</v>
-      </c>
-      <c r="E43" s="17">
-        <v>1</v>
-      </c>
-      <c r="F43" s="17" t="str" cm="1">
-        <f t="array" ref="F43">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E43,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$D$36:$D$47)</f>
-        <v>Rohan + Bhuvanesh</v>
-      </c>
-      <c r="G43" s="24" t="str" cm="1">
-        <f t="array" ref="G43">_xlfn.XLOOKUP("Men's Doubles 2"&amp;E43,'Qualification Data'!$B$36:$B$47&amp;'Qualification Data'!$G$36:$G$47,'Qualification Data'!$C$36:$C$47)</f>
-        <v>Team 6</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A44" s="17"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="24"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A45" s="17"/>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="24"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A46" s="17"/>
-      <c r="B46" s="17"/>
-      <c r="C46" s="17"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
-      <c r="G46" s="24"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A47" s="17"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="24"/>
+      <c r="A38" s="17"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A11:G11"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:G4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G40:G47 G27:G34" xr:uid="{5DB6E15C-AAE4-4337-948C-DFECFF2E6BAE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G34:G38 G27:G31" xr:uid="{5DB6E15C-AAE4-4337-948C-DFECFF2E6BAE}">
       <formula1>"Selected,Not Selected,Pending"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16715,52 +16635,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.15">
-      <c r="A1" s="60" t="s">
+      <c r="A1" s="66" t="s">
         <v>174</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
+      <c r="N1" s="66"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.15">
-      <c r="A2" s="61" t="s">
+      <c r="A2" s="67" t="s">
         <v>248</v>
       </c>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
-      <c r="M2" s="61"/>
-      <c r="N2" s="61"/>
-      <c r="O2" s="61"/>
-      <c r="P2" s="61"/>
-      <c r="Q2" s="61"/>
-      <c r="R2" s="61"/>
-      <c r="S2" s="61"/>
-      <c r="T2" s="61"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="67"/>
+      <c r="M2" s="67"/>
+      <c r="N2" s="67"/>
+      <c r="O2" s="67"/>
+      <c r="P2" s="67"/>
+      <c r="Q2" s="67"/>
+      <c r="R2" s="67"/>
+      <c r="S2" s="67"/>
+      <c r="T2" s="67"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.15">
       <c r="A4" s="49" t="s">
@@ -16849,11 +16769,11 @@
         <v>16</v>
       </c>
       <c r="H5" s="26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" s="26">
         <f t="shared" ref="I5:I20" si="0">IF(OR(F5="",M5=""),"",--(F5&gt;M5)+IF(OR(G5="",N5=""),0,--(G5&gt;N5))+IF(OR(H5="",O5=""),0,--(H5&gt;O5)))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J5" s="27">
         <v>4</v>
@@ -17011,11 +16931,11 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q7" s="28" t="str">
+      <c r="Q7" s="58" t="str">
         <f t="shared" si="2"/>
         <v>Neha P Jain</v>
       </c>
-      <c r="R7" s="28" t="str">
+      <c r="R7" s="58" t="str">
         <f t="shared" si="3"/>
         <v>Team 6</v>
       </c>
@@ -17472,12 +17392,18 @@
         <f>Qualifiers!D28</f>
         <v>Team 3</v>
       </c>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32"/>
-      <c r="H15" s="32"/>
-      <c r="I15" s="32" t="str">
+      <c r="F15" s="32">
+        <v>16</v>
+      </c>
+      <c r="G15" s="32">
+        <v>16</v>
+      </c>
+      <c r="H15" s="32">
+        <v>1</v>
+      </c>
+      <c r="I15" s="32">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="J15" s="33" t="s">
         <v>190</v>
@@ -17490,28 +17416,34 @@
         <f>Qualifiers!G28</f>
         <v>Team 1</v>
       </c>
-      <c r="M15" s="33"/>
-      <c r="N15" s="33"/>
-      <c r="O15" s="33"/>
-      <c r="P15" s="33" t="str">
+      <c r="M15" s="33">
+        <v>7</v>
+      </c>
+      <c r="N15" s="33">
+        <v>11</v>
+      </c>
+      <c r="O15" s="33">
+        <v>0</v>
+      </c>
+      <c r="P15" s="33">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q15" s="31" t="str">
         <f>IF(MAX(N(I15),N(P15))&gt;=2,IF(I15&gt;P15,D15,K15),IF(AND(COUNT(F15:H15,M15:O15)=6,I15=P15),"Tie - review","Pending"))</f>
-        <v>Pending</v>
+        <v>Sujal</v>
       </c>
       <c r="R15" s="31" t="str">
         <f>IF(OR(Q15="Pending",LEFT(Q15,3)="Tie"),Q15,IF(Q15=D15,E15,L15))</f>
-        <v>Pending</v>
-      </c>
-      <c r="S15" s="33" t="str">
+        <v>Team 3</v>
+      </c>
+      <c r="S15" s="33">
         <f>IF(OR(Q15="Pending",LEFT(Q15,3)="Tie"),"",SUMIF('Qualification Data'!$D$23:$D$34,Q15,'Qualification Data'!$F$23:$F$34)+IF(Q15=D15,SUM(F15:H15),SUM(M15:O15)))</f>
-        <v/>
-      </c>
-      <c r="T15" s="33" t="str">
+        <v>131</v>
+      </c>
+      <c r="T15" s="33">
         <f>IF(S15="","",1+COUNTIF($S$14:$S$17,"&gt;"&amp;S15)+COUNTIF($S$14:S15,S15)-1)</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.15">
@@ -17563,11 +17495,11 @@
         <v>16</v>
       </c>
       <c r="O16" s="33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P16" s="33">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q16" s="31" t="str">
         <f>IF(MAX(N(I16),N(P16))&gt;=2,IF(I16&gt;P16,D16,K16),IF(AND(COUNT(F16:H16,M16:O16)=6,I16=P16),"Tie - review","Pending"))</f>
@@ -17579,11 +17511,11 @@
       </c>
       <c r="S16" s="33">
         <f>IF(OR(Q16="Pending",LEFT(Q16,3)="Tie"),"",SUMIF('Qualification Data'!$D$23:$D$34,Q16,'Qualification Data'!$F$23:$F$34)+IF(Q16=D16,SUM(F16:H16),SUM(M16:O16)))</f>
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="T16" s="33">
         <f>IF(S16="","",1+COUNTIF($S$14:$S$17,"&gt;"&amp;S16)+COUNTIF($S$14:S16,S16)-1)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.15">
@@ -17604,12 +17536,18 @@
         <f>Qualifiers!D30</f>
         <v>Team 6</v>
       </c>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
-      <c r="H17" s="32"/>
-      <c r="I17" s="32" t="str">
+      <c r="F17" s="32">
+        <v>5</v>
+      </c>
+      <c r="G17" s="32">
+        <v>6</v>
+      </c>
+      <c r="H17" s="32">
+        <v>0</v>
+      </c>
+      <c r="I17" s="32">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J17" s="33" t="s">
         <v>194</v>
@@ -17622,28 +17560,34 @@
         <f>Qualifiers!G30</f>
         <v>Team 4</v>
       </c>
-      <c r="M17" s="33"/>
-      <c r="N17" s="33"/>
-      <c r="O17" s="33"/>
-      <c r="P17" s="33" t="str">
+      <c r="M17" s="33">
+        <v>16</v>
+      </c>
+      <c r="N17" s="33">
+        <v>16</v>
+      </c>
+      <c r="O17" s="33">
+        <v>1</v>
+      </c>
+      <c r="P17" s="33">
         <f t="shared" si="1"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="Q17" s="31" t="str">
         <f>IF(MAX(N(I17),N(P17))&gt;=2,IF(I17&gt;P17,D17,K17),IF(AND(COUNT(F17:H17,M17:O17)=6,I17=P17),"Tie - review","Pending"))</f>
-        <v>Pending</v>
+        <v>Jay B</v>
       </c>
       <c r="R17" s="31" t="str">
         <f>IF(OR(Q17="Pending",LEFT(Q17,3)="Tie"),Q17,IF(Q17=D17,E17,L17))</f>
-        <v>Pending</v>
-      </c>
-      <c r="S17" s="33" t="str">
+        <v>Team 4</v>
+      </c>
+      <c r="S17" s="33">
         <f>IF(OR(Q17="Pending",LEFT(Q17,3)="Tie"),"",SUMIF('Qualification Data'!$D$23:$D$34,Q17,'Qualification Data'!$F$23:$F$34)+IF(Q17=D17,SUM(F17:H17),SUM(M17:O17)))</f>
-        <v/>
-      </c>
-      <c r="T17" s="33" t="str">
+        <v>138</v>
+      </c>
+      <c r="T17" s="33">
         <f>IF(S17="","",1+COUNTIF($S$14:$S$17,"&gt;"&amp;S17)+COUNTIF($S$14:S17,S17)-1)</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.15">
@@ -17681,8 +17625,8 @@
         <v>Vidwan</v>
       </c>
       <c r="L18" s="27" t="str">
-        <f>IF(K18="TBD","TBD",R16)</f>
-        <v>Team 5</v>
+        <f>IF(K18="TBD","TBD",R15)</f>
+        <v>Team 3</v>
       </c>
       <c r="M18" s="27"/>
       <c r="N18" s="27"/>
@@ -17715,18 +17659,24 @@
       </c>
       <c r="D19" s="25" t="str">
         <f>IF(OR(Q15="Pending",LEFT(Q15,3)="Tie",Q15=""),"TBD",Q15)</f>
-        <v>TBD</v>
+        <v>Sujal</v>
       </c>
       <c r="E19" s="25" t="str">
-        <f>IF(D19="TBD","TBD",R15)</f>
-        <v>TBD</v>
-      </c>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26" t="str">
+        <f>IF(D19="TBD","TBD",R16)</f>
+        <v>Team 5</v>
+      </c>
+      <c r="F19" s="26">
+        <v>9</v>
+      </c>
+      <c r="G19" s="26">
+        <v>9</v>
+      </c>
+      <c r="H19" s="26">
+        <v>0</v>
+      </c>
+      <c r="I19" s="26">
         <f t="shared" si="0"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="J19" s="27" t="str">
         <f>"QF4 Winner"</f>
@@ -17734,26 +17684,32 @@
       </c>
       <c r="K19" s="27" t="str">
         <f>IF(OR(Q17="Pending",LEFT(Q17,3)="Tie",Q17=""),"TBD",Q17)</f>
-        <v>TBD</v>
+        <v>Jay B</v>
       </c>
       <c r="L19" s="27" t="str">
         <f>IF(K19="TBD","TBD",R17)</f>
-        <v>TBD</v>
-      </c>
-      <c r="M19" s="27"/>
-      <c r="N19" s="27"/>
-      <c r="O19" s="27"/>
-      <c r="P19" s="27" t="str">
+        <v>Team 4</v>
+      </c>
+      <c r="M19" s="27">
+        <v>16</v>
+      </c>
+      <c r="N19" s="27">
+        <v>16</v>
+      </c>
+      <c r="O19" s="27">
+        <v>1</v>
+      </c>
+      <c r="P19" s="27">
         <f t="shared" si="1"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="Q19" s="25" t="str">
         <f t="shared" si="2"/>
-        <v>Pending</v>
+        <v>Jay B</v>
       </c>
       <c r="R19" s="25" t="str">
         <f t="shared" si="3"/>
-        <v>Pending</v>
+        <v>Team 4</v>
       </c>
       <c r="S19" s="27"/>
       <c r="T19" s="27"/>
@@ -17788,11 +17744,11 @@
       </c>
       <c r="K20" s="30" t="str">
         <f>IF(OR(Q19="Pending",LEFT(Q19,3)="Tie"),"TBD",Q19)</f>
-        <v>TBD</v>
+        <v>Jay B</v>
       </c>
       <c r="L20" s="30" t="str">
         <f>IF(OR(R19="Pending",LEFT(R19,3)="Tie"),"TBD",R19)</f>
-        <v>TBD</v>
+        <v>Team 4</v>
       </c>
       <c r="M20" s="30"/>
       <c r="N20" s="30"/>
@@ -17845,11 +17801,11 @@
         <v>195</v>
       </c>
       <c r="D22" s="31" t="str">
-        <f>Qualifiers!C40</f>
+        <f>Qualifiers!C34</f>
         <v>Kushal + Shubham</v>
       </c>
       <c r="E22" s="31" t="str">
-        <f>Qualifiers!D40</f>
+        <f>Qualifiers!D34</f>
         <v>Team 2</v>
       </c>
       <c r="F22" s="32"/>
@@ -17863,11 +17819,11 @@
         <v>196</v>
       </c>
       <c r="K22" s="33" t="str">
-        <f>Qualifiers!F40</f>
+        <f>Qualifiers!F34</f>
         <v>Khush B + Hemanth</v>
       </c>
       <c r="L22" s="33" t="str">
-        <f>Qualifiers!G40</f>
+        <f>Qualifiers!G34</f>
         <v>Team 4</v>
       </c>
       <c r="M22" s="33"/>
@@ -17905,53 +17861,65 @@
         <v>197</v>
       </c>
       <c r="D23" s="31" t="str">
-        <f>Qualifiers!C41</f>
+        <f>Qualifiers!C35</f>
         <v>Kunal D + Anirudha H</v>
       </c>
       <c r="E23" s="31" t="str">
-        <f>Qualifiers!D41</f>
+        <f>Qualifiers!D35</f>
         <v>Team 3</v>
       </c>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
-      <c r="H23" s="32"/>
-      <c r="I23" s="32" t="str">
+      <c r="F23" s="32">
+        <v>16</v>
+      </c>
+      <c r="G23" s="32">
+        <v>18</v>
+      </c>
+      <c r="H23" s="32">
+        <v>1</v>
+      </c>
+      <c r="I23" s="32">
         <f t="shared" si="4"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="J23" s="33" t="s">
         <v>198</v>
       </c>
       <c r="K23" s="33" t="str">
-        <f>Qualifiers!F41</f>
+        <f>Qualifiers!F35</f>
         <v>Yuvraj + Karthik KB</v>
       </c>
       <c r="L23" s="33" t="str">
-        <f>Qualifiers!G41</f>
+        <f>Qualifiers!G35</f>
         <v>Team 2</v>
       </c>
-      <c r="M23" s="33"/>
-      <c r="N23" s="33"/>
-      <c r="O23" s="33"/>
-      <c r="P23" s="33" t="str">
+      <c r="M23" s="33">
+        <v>10</v>
+      </c>
+      <c r="N23" s="33">
+        <v>17</v>
+      </c>
+      <c r="O23" s="33">
+        <v>0</v>
+      </c>
+      <c r="P23" s="33">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q23" s="31" t="str">
         <f>IF(MAX(N(I23),N(P23))&gt;=2,IF(I23&gt;P23,D23,K23),IF(AND(COUNT(F23:H23,M23:O23)=6,I23=P23),"Tie - review","Pending"))</f>
-        <v>Pending</v>
+        <v>Kunal D + Anirudha H</v>
       </c>
       <c r="R23" s="31" t="str">
         <f>IF(OR(Q23="Pending",LEFT(Q23,3)="Tie"),Q23,IF(Q23=D23,E23,L23))</f>
-        <v>Pending</v>
-      </c>
-      <c r="S23" s="33" t="str">
+        <v>Team 3</v>
+      </c>
+      <c r="S23" s="33">
         <f>IF(OR(Q23="Pending",LEFT(Q23,3)="Tie"),"",SUMIF('Qualification Data'!$D$36:$D$47,Q23,'Qualification Data'!$F$36:$F$47)+IF(Q23=D23,SUM(F23:H23),SUM(M23:O23)))</f>
-        <v/>
-      </c>
-      <c r="T23" s="33" t="str">
+        <v>135</v>
+      </c>
+      <c r="T23" s="33">
         <f>IF(S23="","",1+COUNTIF($S$22:$S$25,"&gt;"&amp;S23)+COUNTIF($S$22:S23,S23)-1)</f>
-        <v/>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.15">
@@ -17965,11 +17933,11 @@
         <v>199</v>
       </c>
       <c r="D24" s="31" t="str">
-        <f>Qualifiers!C42</f>
+        <f>Qualifiers!C36</f>
         <v>Leela Sagar + Ali Akbar</v>
       </c>
       <c r="E24" s="31" t="str">
-        <f>Qualifiers!D42</f>
+        <f>Qualifiers!D36</f>
         <v>Team 4</v>
       </c>
       <c r="F24" s="32">
@@ -17989,11 +17957,11 @@
         <v>200</v>
       </c>
       <c r="K24" s="33" t="str">
-        <f>Qualifiers!F42</f>
+        <f>Qualifiers!F36</f>
         <v>Sarvesh H + Deviprasad</v>
       </c>
       <c r="L24" s="33" t="str">
-        <f>Qualifiers!G42</f>
+        <f>Qualifiers!G36</f>
         <v>Team 3</v>
       </c>
       <c r="M24" s="33">
@@ -18037,11 +18005,11 @@
         <v>201</v>
       </c>
       <c r="D25" s="31" t="str">
-        <f>Qualifiers!C43</f>
+        <f>Qualifiers!C37</f>
         <v>Nagarajan + Chandrashaker Joshi</v>
       </c>
       <c r="E25" s="31" t="str">
-        <f>Qualifiers!D43</f>
+        <f>Qualifiers!D37</f>
         <v>Team 6</v>
       </c>
       <c r="F25" s="32">
@@ -18051,21 +18019,21 @@
         <v>16</v>
       </c>
       <c r="H25" s="32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" s="32">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J25" s="33" t="s">
         <v>202</v>
       </c>
       <c r="K25" s="33" t="str">
-        <f>Qualifiers!F43</f>
+        <f>Qualifiers!F37</f>
         <v>Rohan + Bhuvanesh</v>
       </c>
       <c r="L25" s="33" t="str">
-        <f>Qualifiers!G43</f>
+        <f>Qualifiers!G37</f>
         <v>Team 6</v>
       </c>
       <c r="M25" s="33">
@@ -18091,11 +18059,11 @@
       </c>
       <c r="S25" s="33">
         <f>IF(OR(Q25="Pending",LEFT(Q25,3)="Tie"),"",SUMIF('Qualification Data'!$D$36:$D$47,Q25,'Qualification Data'!$F$36:$F$47)+IF(Q25=D25,SUM(F25:H25),SUM(M25:O25)))</f>
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="T25" s="33">
         <f>IF(S25="","",1+COUNTIF($S$22:$S$25,"&gt;"&amp;S25)+COUNTIF($S$22:S25,S25)-1)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.15">
@@ -18133,7 +18101,7 @@
         <v>Sarvesh H + Deviprasad</v>
       </c>
       <c r="L26" s="27" t="str">
-        <f>IF(K26="TBD","TBD",R24)</f>
+        <f>IF(K26="TBD","TBD",R23)</f>
         <v>Team 3</v>
       </c>
       <c r="M26" s="27"/>
@@ -18162,16 +18130,16 @@
         <v>183</v>
       </c>
       <c r="C27" s="25" t="str">
-        <f>"QF2 Winner"</f>
-        <v>QF2 Winner</v>
+        <f>"QF4 Winner"</f>
+        <v>QF4 Winner</v>
       </c>
       <c r="D27" s="25" t="str">
         <f>IF(OR(Q23="Pending",LEFT(Q23,3)="Tie",Q23=""),"TBD",Q23)</f>
-        <v>TBD</v>
+        <v>Kunal D + Anirudha H</v>
       </c>
       <c r="E27" s="25" t="str">
-        <f>IF(D27="TBD","TBD",R23)</f>
-        <v>TBD</v>
+        <f>IF(D27="TBD","TBD",R24)</f>
+        <v>Team 3</v>
       </c>
       <c r="F27" s="26"/>
       <c r="G27" s="26"/>
@@ -18288,20 +18256,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="64" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-    </row>
-    <row r="2" spans="1:10" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="64"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A2" s="68" t="s">
         <v>246</v>
       </c>
@@ -18438,7 +18406,7 @@
       </c>
       <c r="J6" s="36">
         <f t="shared" ref="J6:J10" si="4">_xlfn.RANK.EQ(I6,$I$5:$I$10,0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.15">
@@ -18451,11 +18419,11 @@
       </c>
       <c r="C7" s="35">
         <f>SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A7,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A7,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A7,Finals!$B$5:$B$28,"Semifinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A7,Finals!$B$5:$B$28,"Semifinal*")</f>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D7" s="35">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E7" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A7,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
@@ -18475,11 +18443,11 @@
       </c>
       <c r="I7" s="36">
         <f t="shared" si="3"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="J7" s="36">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="48" customFormat="1" x14ac:dyDescent="0.15">
@@ -18492,11 +18460,11 @@
       </c>
       <c r="C8" s="35">
         <f>SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A8,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A8,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A8,Finals!$B$5:$B$28,"Semifinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A8,Finals!$B$5:$B$28,"Semifinal*")</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D8" s="35">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E8" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A8,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
@@ -18516,11 +18484,11 @@
       </c>
       <c r="I8" s="36">
         <f t="shared" si="3"/>
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="J8" s="36">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.15">
@@ -18533,11 +18501,11 @@
       </c>
       <c r="C9" s="35">
         <f>SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A9,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A9,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A9,Finals!$B$5:$B$28,"Semifinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A9,Finals!$B$5:$B$28,"Semifinal*")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="35">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A9,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
@@ -18557,7 +18525,7 @@
       </c>
       <c r="I9" s="36">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J9" s="36">
         <f t="shared" si="4"/>
@@ -18574,11 +18542,11 @@
       </c>
       <c r="C10" s="35">
         <f>SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A10,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A10,Finals!$B$5:$B$28,"Quarterfinal*")+SUMIFS(Finals!$I$5:$I$28,Finals!$E$5:$E$28,$A10,Finals!$B$5:$B$28,"Semifinal*")+SUMIFS(Finals!$P$5:$P$28,Finals!$L$5:$L$28,$A10,Finals!$B$5:$B$28,"Semifinal*")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D10" s="35">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E10" s="35">
         <f>COUNTIFS(Finals!$B$5:$B$28,"Final",Finals!$R$5:$R$28,$A10,Finals!$E$5:$E$28,"Team*",Finals!$L$5:$L$28,"Team*")</f>
@@ -18598,7 +18566,7 @@
       </c>
       <c r="I10" s="36">
         <f t="shared" si="3"/>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J10" s="36">
         <f t="shared" si="4"/>

</xml_diff>